<commit_message>
chore: sync qt monitor source and yolo tools
</commit_message>
<xml_diff>
--- a/docs/进度跟踪表.xlsx
+++ b/docs/进度跟踪表.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\qt6code\day20\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="25596" windowHeight="12095"/>
+    <workbookView windowWidth="30720" windowHeight="13380"/>
   </bookViews>
   <sheets>
     <sheet name="进度规划表" sheetId="1" r:id="rId1"/>
@@ -510,7 +515,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -544,6 +549,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -924,7 +935,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -948,16 +959,16 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -966,90 +977,90 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1087,19 +1098,34 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="30" fontId="1" fillId="7" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="30" fontId="4" fillId="7" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="30" fontId="1" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1864,10 +1890,10 @@
       <c r="D13" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="14">
+      <c r="F13" s="15">
         <v>46221</v>
       </c>
       <c r="G13" s="7" t="s">
@@ -1879,13 +1905,13 @@
         <v>11</v>
       </c>
       <c r="C14" s="12"/>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="15">
         <v>46221</v>
       </c>
       <c r="G14" s="11" t="s">
@@ -2007,17 +2033,17 @@
         <v>18</v>
       </c>
       <c r="C21" s="12"/>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="F21" s="14">
+      <c r="F21" s="15">
         <v>46222</v>
       </c>
-      <c r="G21" s="11" t="s">
-        <v>4</v>
+      <c r="G21" s="7" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1" spans="2:7">
@@ -2025,13 +2051,13 @@
         <v>19</v>
       </c>
       <c r="C22" s="8"/>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="F22" s="10">
+      <c r="F22" s="17">
         <v>46222</v>
       </c>
       <c r="G22" s="7" t="s">
@@ -2043,16 +2069,16 @@
         <v>20</v>
       </c>
       <c r="C23" s="12"/>
-      <c r="D23" s="13" t="s">
+      <c r="D23" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="F23" s="14">
+      <c r="F23" s="15">
         <v>46222</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="G23" s="7" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2073,7 +2099,7 @@
         <v>46223</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="21" customHeight="1" spans="2:7">
@@ -2081,17 +2107,17 @@
         <v>22</v>
       </c>
       <c r="C25" s="12"/>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="F25" s="14">
+      <c r="F25" s="15">
         <v>46223</v>
       </c>
-      <c r="G25" s="11" t="s">
-        <v>4</v>
+      <c r="G25" s="7" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="26" ht="21" customHeight="1" spans="2:7">
@@ -2099,17 +2125,17 @@
         <v>23</v>
       </c>
       <c r="C26" s="8"/>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="F26" s="10">
+      <c r="F26" s="17">
         <v>46223</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="21" customHeight="1" spans="2:7">
@@ -2117,17 +2143,17 @@
         <v>24</v>
       </c>
       <c r="C27" s="8"/>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="F27" s="10">
+      <c r="F27" s="17">
         <v>46223</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" ht="21" customHeight="1" spans="2:7">
@@ -2135,17 +2161,17 @@
         <v>25</v>
       </c>
       <c r="C28" s="12"/>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="F28" s="14">
+      <c r="F28" s="15">
         <v>46223</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" ht="21" customHeight="1" spans="2:7">
@@ -2163,7 +2189,7 @@
         <v>46223</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="21" customHeight="1" spans="2:7">
@@ -2183,7 +2209,7 @@
         <v>46224</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="21" customHeight="1" spans="2:7">
@@ -2201,7 +2227,7 @@
         <v>46224</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="21" customHeight="1" spans="2:7">
@@ -2219,7 +2245,7 @@
         <v>46224</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="21" customHeight="1" spans="2:7">
@@ -2237,7 +2263,7 @@
         <v>46224</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" ht="21" customHeight="1" spans="2:7">
@@ -2255,7 +2281,7 @@
         <v>46224</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="21" customHeight="1" spans="2:7">
@@ -2263,17 +2289,17 @@
         <v>32</v>
       </c>
       <c r="C35" s="12"/>
-      <c r="D35" s="13" t="s">
+      <c r="D35" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E35" s="13" t="s">
+      <c r="E35" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="F35" s="14">
+      <c r="F35" s="19">
         <v>46224</v>
       </c>
-      <c r="G35" s="11" t="s">
-        <v>4</v>
+      <c r="G35" s="7" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="36" ht="21" customHeight="1" spans="2:7">
@@ -2293,7 +2319,7 @@
         <v>46225</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="21" customHeight="1" spans="2:7">
@@ -2301,17 +2327,17 @@
         <v>34</v>
       </c>
       <c r="C37" s="12"/>
-      <c r="D37" s="13" t="s">
+      <c r="D37" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="E37" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="F37" s="14">
+      <c r="F37" s="19">
         <v>46225</v>
       </c>
-      <c r="G37" s="11" t="s">
-        <v>4</v>
+      <c r="G37" s="7" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="21" customHeight="1" spans="2:7">
@@ -2319,13 +2345,13 @@
         <v>35</v>
       </c>
       <c r="C38" s="12"/>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E38" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="F38" s="14">
+      <c r="F38" s="19">
         <v>46225</v>
       </c>
       <c r="G38" s="11" t="s">
@@ -2369,12 +2395,12 @@
       </c>
     </row>
     <row r="41" ht="18" customHeight="1" spans="2:7">
-      <c r="B41" s="15"/>
-      <c r="C41" s="16"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
-      <c r="F41" s="16"/>
-      <c r="G41" s="17"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2408,7 +2434,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="G14 G4:G5 G6:G13 G15:G20 G21:G40">
+    <dataValidation type="list" sqref="G4:G19 G20:G26 G27:G28 G29:G37 G38:G40">
       <formula1>"未开始,进行中,已完成,风险"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>